<commit_message>
Stop tracking virtual environment
</commit_message>
<xml_diff>
--- a/dataset_making/master.xlsx
+++ b/dataset_making/master.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD3"/>
+  <dimension ref="A1:AE10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -579,15 +579,20 @@
           <t>wrist_speed_at_release_m_s</t>
         </is>
       </c>
+      <c r="AE1" s="1" t="inlineStr">
+        <is>
+          <t>release_method</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>new</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>59.97095837366893</v>
+        <v>59.96430696014277</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -600,88 +605,93 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>408</v>
+        <v>149</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>[291, 316, 348, 401, 401]</t>
+          <t>[87, 118, 135, 143, 149]</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>[0.41686844229217107, 0.533591606133979, 0.8837610976594027, 0.0]</t>
+          <t>[0.5169742063492063, 0.28350198412698413, 0.13341269841269843, 0.1000595238095238]</t>
         </is>
       </c>
       <c r="H2" t="n">
-        <v>0.4585552865213882</v>
+        <v>0.2584871031746032</v>
       </c>
       <c r="I2" t="n">
-        <v>0.3156109847838963</v>
+        <v>0.1644568571135626</v>
       </c>
       <c r="J2" t="n">
-        <v>0.6882724811180981</v>
+        <v>0.6362284813972909</v>
       </c>
       <c r="K2" t="n">
-        <v>1.834221146085553</v>
+        <v>1.033948412698413</v>
       </c>
       <c r="L2" t="n">
-        <v>0.4335431799838579</v>
+        <v>0.1000595238095238</v>
       </c>
       <c r="M2" t="n">
-        <v>0.3191826601565718</v>
+        <v>0.8622171134760422</v>
       </c>
       <c r="N2" t="n">
-        <v>375</v>
+        <v>143</v>
       </c>
       <c r="O2" t="n">
-        <v>401</v>
+        <v>149</v>
       </c>
       <c r="P2" t="n">
-        <v>401</v>
+        <v>141</v>
       </c>
       <c r="Q2" t="n">
-        <v>408</v>
+        <v>149</v>
       </c>
       <c r="R2" t="n">
-        <v>170.5578369948597</v>
+        <v>139.015577024508</v>
       </c>
       <c r="S2" t="inlineStr"/>
       <c r="T2" t="inlineStr"/>
-      <c r="U2" t="inlineStr"/>
-      <c r="V2" t="inlineStr"/>
+      <c r="U2" t="n">
+        <v>142.9280982007073</v>
+      </c>
+      <c r="V2" t="n">
+        <v>142.9280982007073</v>
+      </c>
       <c r="W2" t="n">
-        <v>-256.8290392545429</v>
+        <v>-562.4669483176417</v>
       </c>
       <c r="X2" t="n">
-        <v>-167.7548004341224</v>
+        <v>-237.3654033305984</v>
       </c>
       <c r="Y2" t="n">
-        <v>306.761843248315</v>
+        <v>610.5009440189739</v>
       </c>
       <c r="Z2" t="n">
-        <v>-194.2102282909209</v>
+        <v>-157.433501399148</v>
       </c>
       <c r="AA2" t="n">
-        <v>-156.8099907686192</v>
+        <v>-163.4324389536099</v>
       </c>
       <c r="AB2" t="n">
-        <v>249.6136734589394</v>
+        <v>226.9261321776779</v>
       </c>
       <c r="AC2" t="n">
-        <v>92.1884208810102</v>
+        <v>85.7056358273985</v>
       </c>
       <c r="AD2" t="n">
-        <v>28.1971264084378</v>
-      </c>
+        <v>38.80394992768173</v>
+      </c>
+      <c r="AE2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3051f922</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>59.96430696014277</v>
+        <v>60</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -694,83 +704,809 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>149</v>
+        <v>229</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>[87, 118, 135, 143, 149]</t>
+          <t>[102, 125, 143, 185, 222]</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>[0.5169742063492063, 0.28350198412698413, 0.13341269841269843, 0.1000595238095238]</t>
+          <t>[0.38333333333333336, 0.3, 0.7, 0.6166666666666667]</t>
         </is>
       </c>
       <c r="H3" t="n">
-        <v>0.2584871031746032</v>
+        <v>0.5</v>
       </c>
       <c r="I3" t="n">
-        <v>0.1644568571135626</v>
+        <v>0.1637240225365708</v>
       </c>
       <c r="J3" t="n">
-        <v>0.6362284813972909</v>
+        <v>0.3274480450731416</v>
       </c>
       <c r="K3" t="n">
-        <v>1.033948412698413</v>
+        <v>2</v>
       </c>
       <c r="L3" t="n">
-        <v>0.1000595238095238</v>
+        <v>0.6166666666666667</v>
       </c>
       <c r="M3" t="n">
-        <v>0.8622171134760422</v>
+        <v>0.6542775424299568</v>
       </c>
       <c r="N3" t="n">
-        <v>143</v>
+        <v>185</v>
       </c>
       <c r="O3" t="n">
-        <v>149</v>
+        <v>222</v>
       </c>
       <c r="P3" t="n">
-        <v>141</v>
+        <v>225</v>
       </c>
       <c r="Q3" t="n">
-        <v>149</v>
+        <v>229</v>
       </c>
       <c r="R3" t="n">
-        <v>139.015577024508</v>
-      </c>
-      <c r="S3" t="inlineStr"/>
-      <c r="T3" t="inlineStr"/>
+        <v>159.9886405983499</v>
+      </c>
+      <c r="S3" t="n">
+        <v>165.9477119898054</v>
+      </c>
+      <c r="T3" t="n">
+        <v>5.95907139145541</v>
+      </c>
       <c r="U3" t="n">
-        <v>142.9280982007073</v>
+        <v>147.6960441740065</v>
       </c>
       <c r="V3" t="n">
-        <v>142.9280982007073</v>
+        <v>173.5375067144464</v>
       </c>
       <c r="W3" t="n">
-        <v>-562.4669483176417</v>
+        <v>-233.2376728852371</v>
       </c>
       <c r="X3" t="n">
-        <v>-237.3654033305984</v>
+        <v>-195.8683052262931</v>
       </c>
       <c r="Y3" t="n">
-        <v>610.5009440189739</v>
+        <v>304.5721672200879</v>
       </c>
       <c r="Z3" t="n">
-        <v>-157.433501399148</v>
+        <v>-157.154503670528</v>
       </c>
       <c r="AA3" t="n">
-        <v>-163.4324389536099</v>
+        <v>-178.741332149111</v>
       </c>
       <c r="AB3" t="n">
-        <v>226.9261321776779</v>
+        <v>238.0042055140388</v>
       </c>
       <c r="AC3" t="n">
-        <v>85.7056358273985</v>
+        <v>88.1173863413308</v>
       </c>
       <c r="AD3" t="n">
-        <v>38.80394992768173</v>
-      </c>
+        <v>88.1173863413308</v>
+      </c>
+      <c r="AE3" t="inlineStr">
+        <is>
+          <t>wrist_speed_peak_drop</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>324e1188</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>60</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>SIDE</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>144</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>[39, 60, 74, 104, 126]</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>[0.35, 0.23333333333333334, 0.5, 0.36666666666666664]</t>
+        </is>
+      </c>
+      <c r="H4" t="n">
+        <v>0.3625</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0.09455671431591847</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0.2608461084577061</v>
+      </c>
+      <c r="K4" t="n">
+        <v>1.45</v>
+      </c>
+      <c r="L4" t="n">
+        <v>0.3666666666666666</v>
+      </c>
+      <c r="M4" t="n">
+        <v>0.9290980777877696</v>
+      </c>
+      <c r="N4" t="n">
+        <v>104</v>
+      </c>
+      <c r="O4" t="n">
+        <v>126</v>
+      </c>
+      <c r="P4" t="n">
+        <v>134</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>144</v>
+      </c>
+      <c r="R4" t="n">
+        <v>146.2370153336146</v>
+      </c>
+      <c r="S4" t="n">
+        <v>90.80948260711824</v>
+      </c>
+      <c r="T4" t="n">
+        <v>-55.42753272649634</v>
+      </c>
+      <c r="U4" t="inlineStr"/>
+      <c r="V4" t="inlineStr"/>
+      <c r="W4" t="n">
+        <v>-176.5019353150292</v>
+      </c>
+      <c r="X4" t="n">
+        <v>-161.3347266415383</v>
+      </c>
+      <c r="Y4" t="n">
+        <v>239.1272196769968</v>
+      </c>
+      <c r="Z4" t="n">
+        <v>-232.3055980567109</v>
+      </c>
+      <c r="AA4" t="n">
+        <v>-169.8306428187528</v>
+      </c>
+      <c r="AB4" t="n">
+        <v>287.764379534224</v>
+      </c>
+      <c r="AC4" t="n">
+        <v>50.532376796942</v>
+      </c>
+      <c r="AD4" t="n">
+        <v>50.532376796942</v>
+      </c>
+      <c r="AE4" t="inlineStr">
+        <is>
+          <t>wrist_speed_peak_drop</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>5296fd61</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>60</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>SIDE</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>172</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>[66, 102, 115, 140, 159]</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>[0.6, 0.21666666666666667, 0.4166666666666667, 0.31666666666666665]</t>
+        </is>
+      </c>
+      <c r="H5" t="n">
+        <v>0.3875</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0.1416053788997202</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0.3654332358702457</v>
+      </c>
+      <c r="K5" t="n">
+        <v>1.55</v>
+      </c>
+      <c r="L5" t="n">
+        <v>0.3166666666666667</v>
+      </c>
+      <c r="M5" t="n">
+        <v>1.014399664938039</v>
+      </c>
+      <c r="N5" t="n">
+        <v>140</v>
+      </c>
+      <c r="O5" t="n">
+        <v>159</v>
+      </c>
+      <c r="P5" t="n">
+        <v>168</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>172</v>
+      </c>
+      <c r="R5" t="n">
+        <v>130.120654017213</v>
+      </c>
+      <c r="S5" t="n">
+        <v>170.9802080620529</v>
+      </c>
+      <c r="T5" t="n">
+        <v>40.85955404483991</v>
+      </c>
+      <c r="U5" t="n">
+        <v>153.169707840219</v>
+      </c>
+      <c r="V5" t="n">
+        <v>172.1998032540796</v>
+      </c>
+      <c r="W5" t="n">
+        <v>-162.964036402209</v>
+      </c>
+      <c r="X5" t="n">
+        <v>-205.9193725922683</v>
+      </c>
+      <c r="Y5" t="n">
+        <v>262.6024850782908</v>
+      </c>
+      <c r="Z5" t="n">
+        <v>-131.3963083917026</v>
+      </c>
+      <c r="AA5" t="n">
+        <v>-180.9027141281654</v>
+      </c>
+      <c r="AB5" t="n">
+        <v>223.5861843627735</v>
+      </c>
+      <c r="AC5" t="n">
+        <v>66.28715163020401</v>
+      </c>
+      <c r="AD5" t="n">
+        <v>66.28715163020401</v>
+      </c>
+      <c r="AE5" t="inlineStr">
+        <is>
+          <t>wrist_speed_peak_drop</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>68372319</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>60</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>SIDE</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>188</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>[83, 101, 118, 148, 172]</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>[0.3, 0.2833333333333333, 0.5, 0.4]</t>
+        </is>
+      </c>
+      <c r="H6" t="n">
+        <v>0.3708333333333333</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0.08690272339422588</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0.2343444226361147</v>
+      </c>
+      <c r="K6" t="n">
+        <v>1.483333333333333</v>
+      </c>
+      <c r="L6" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="M6" t="n">
+        <v>1.140319775390625</v>
+      </c>
+      <c r="N6" t="n">
+        <v>148</v>
+      </c>
+      <c r="O6" t="n">
+        <v>172</v>
+      </c>
+      <c r="P6" t="n">
+        <v>176</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>188</v>
+      </c>
+      <c r="R6" t="n">
+        <v>148.6978025554788</v>
+      </c>
+      <c r="S6" t="inlineStr"/>
+      <c r="T6" t="inlineStr"/>
+      <c r="U6" t="inlineStr"/>
+      <c r="V6" t="inlineStr"/>
+      <c r="W6" t="n">
+        <v>-167.1142939453125</v>
+      </c>
+      <c r="X6" t="n">
+        <v>-162.4537924804687</v>
+      </c>
+      <c r="Y6" t="n">
+        <v>233.0631286414209</v>
+      </c>
+      <c r="Z6" t="n">
+        <v>-141.93495703125</v>
+      </c>
+      <c r="AA6" t="n">
+        <v>-156.7751451416015</v>
+      </c>
+      <c r="AB6" t="n">
+        <v>211.4804439224417</v>
+      </c>
+      <c r="AC6" t="n">
+        <v>91.81127061619543</v>
+      </c>
+      <c r="AD6" t="n">
+        <v>91.81127061619543</v>
+      </c>
+      <c r="AE6" t="inlineStr">
+        <is>
+          <t>wrist_speed_peak_drop</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>93a73e01</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>60</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>SIDE</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>144</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>[39, 60, 74, 104, 126]</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>[0.35, 0.23333333333333334, 0.5, 0.36666666666666664]</t>
+        </is>
+      </c>
+      <c r="H7" t="n">
+        <v>0.3625</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0.09455671431591847</v>
+      </c>
+      <c r="J7" t="n">
+        <v>0.2608461084577061</v>
+      </c>
+      <c r="K7" t="n">
+        <v>1.45</v>
+      </c>
+      <c r="L7" t="n">
+        <v>0.3666666666666666</v>
+      </c>
+      <c r="M7" t="n">
+        <v>0.983334767607868</v>
+      </c>
+      <c r="N7" t="n">
+        <v>104</v>
+      </c>
+      <c r="O7" t="n">
+        <v>126</v>
+      </c>
+      <c r="P7" t="n">
+        <v>134</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>144</v>
+      </c>
+      <c r="R7" t="n">
+        <v>146.2370153336146</v>
+      </c>
+      <c r="S7" t="n">
+        <v>90.80948260711824</v>
+      </c>
+      <c r="T7" t="n">
+        <v>-55.42753272649634</v>
+      </c>
+      <c r="U7" t="inlineStr"/>
+      <c r="V7" t="inlineStr"/>
+      <c r="W7" t="n">
+        <v>-186.8053477826579</v>
+      </c>
+      <c r="X7" t="n">
+        <v>-170.7527436789885</v>
+      </c>
+      <c r="Y7" t="n">
+        <v>253.0864228561108</v>
+      </c>
+      <c r="Z7" t="n">
+        <v>-245.8665847453006</v>
+      </c>
+      <c r="AA7" t="n">
+        <v>-179.7446143538577</v>
+      </c>
+      <c r="AB7" t="n">
+        <v>304.5628077811456</v>
+      </c>
+      <c r="AC7" t="n">
+        <v>53.48223635615436</v>
+      </c>
+      <c r="AD7" t="n">
+        <v>53.48223635615436</v>
+      </c>
+      <c r="AE7" t="inlineStr">
+        <is>
+          <t>wrist_speed_peak_drop</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Ravien</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>60</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>SIDE</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>137</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>[48, 64, 93, 113, 117]</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>[0.26666666666666666, 0.48333333333333334, 0.3333333333333333, 0.06666666666666667]</t>
+        </is>
+      </c>
+      <c r="H8" t="n">
+        <v>0.2875</v>
+      </c>
+      <c r="I8" t="n">
+        <v>0.1497103685268474</v>
+      </c>
+      <c r="J8" t="n">
+        <v>0.5207317166151213</v>
+      </c>
+      <c r="K8" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="L8" t="n">
+        <v>0.06666666666666667</v>
+      </c>
+      <c r="M8" t="n">
+        <v>0.3948693544708029</v>
+      </c>
+      <c r="N8" t="n">
+        <v>113</v>
+      </c>
+      <c r="O8" t="n">
+        <v>117</v>
+      </c>
+      <c r="P8" t="n">
+        <v>133</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>137</v>
+      </c>
+      <c r="R8" t="n">
+        <v>141.8835715327521</v>
+      </c>
+      <c r="S8" t="n">
+        <v>114.2584639841698</v>
+      </c>
+      <c r="T8" t="n">
+        <v>-27.62510754858228</v>
+      </c>
+      <c r="U8" t="n">
+        <v>120.9587913280582</v>
+      </c>
+      <c r="V8" t="n">
+        <v>147.0618184763749</v>
+      </c>
+      <c r="W8" t="n">
+        <v>-405.1679359959512</v>
+      </c>
+      <c r="X8" t="n">
+        <v>-238.2634633397012</v>
+      </c>
+      <c r="Y8" t="n">
+        <v>470.0324821986756</v>
+      </c>
+      <c r="Z8" t="n">
+        <v>-211.5529426608121</v>
+      </c>
+      <c r="AA8" t="n">
+        <v>-188.4309182004163</v>
+      </c>
+      <c r="AB8" t="n">
+        <v>283.3034741797227</v>
+      </c>
+      <c r="AC8" t="n">
+        <v>68.02571630402693</v>
+      </c>
+      <c r="AD8" t="n">
+        <v>68.02571630402693</v>
+      </c>
+      <c r="AE8" t="inlineStr">
+        <is>
+          <t>wrist_speed_peak_drop</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Ravien 2</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>60</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>SIDE</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>200</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>[88, 108, 162, 163, 192]</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>[0.3333333333333333, 0.9, 0.016666666666666666, 0.48333333333333334]</t>
+        </is>
+      </c>
+      <c r="H9" t="n">
+        <v>0.4333333333333333</v>
+      </c>
+      <c r="I9" t="n">
+        <v>0.3177612660822937</v>
+      </c>
+      <c r="J9" t="n">
+        <v>0.7332952294206776</v>
+      </c>
+      <c r="K9" t="n">
+        <v>1.733333333333334</v>
+      </c>
+      <c r="L9" t="n">
+        <v>0.4833333333333333</v>
+      </c>
+      <c r="M9" t="n">
+        <v>1.069224948584209</v>
+      </c>
+      <c r="N9" t="n">
+        <v>163</v>
+      </c>
+      <c r="O9" t="n">
+        <v>192</v>
+      </c>
+      <c r="P9" t="n">
+        <v>196</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>200</v>
+      </c>
+      <c r="R9" t="n">
+        <v>135.3284782964824</v>
+      </c>
+      <c r="S9" t="n">
+        <v>148.9634442714724</v>
+      </c>
+      <c r="T9" t="n">
+        <v>13.63496597498997</v>
+      </c>
+      <c r="U9" t="inlineStr"/>
+      <c r="V9" t="inlineStr"/>
+      <c r="W9" t="n">
+        <v>-170.7379109663018</v>
+      </c>
+      <c r="X9" t="n">
+        <v>-161.0690270602319</v>
+      </c>
+      <c r="Y9" t="n">
+        <v>234.722529211123</v>
+      </c>
+      <c r="Z9" t="n">
+        <v>-224.0349215487291</v>
+      </c>
+      <c r="AA9" t="n">
+        <v>-169.0981742556524</v>
+      </c>
+      <c r="AB9" t="n">
+        <v>280.6881518873573</v>
+      </c>
+      <c r="AC9" t="n">
+        <v>79.74137467015595</v>
+      </c>
+      <c r="AD9" t="n">
+        <v>79.74137467015595</v>
+      </c>
+      <c r="AE9" t="inlineStr">
+        <is>
+          <t>wrist_speed_peak_drop</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>59.97095837366893</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>SIDE</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>408</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>[291, 316, 348, 401, 401]</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>[0.41686844229217107, 0.533591606133979, 0.8837610976594027, 0.0]</t>
+        </is>
+      </c>
+      <c r="H10" t="n">
+        <v>0.4585552865213882</v>
+      </c>
+      <c r="I10" t="n">
+        <v>0.3156109847838963</v>
+      </c>
+      <c r="J10" t="n">
+        <v>0.6882724811180981</v>
+      </c>
+      <c r="K10" t="n">
+        <v>1.834221146085553</v>
+      </c>
+      <c r="L10" t="n">
+        <v>0.4335431799838579</v>
+      </c>
+      <c r="M10" t="n">
+        <v>0.3191826601565718</v>
+      </c>
+      <c r="N10" t="n">
+        <v>375</v>
+      </c>
+      <c r="O10" t="n">
+        <v>401</v>
+      </c>
+      <c r="P10" t="n">
+        <v>401</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>408</v>
+      </c>
+      <c r="R10" t="n">
+        <v>170.5578369948597</v>
+      </c>
+      <c r="S10" t="inlineStr"/>
+      <c r="T10" t="inlineStr"/>
+      <c r="U10" t="inlineStr"/>
+      <c r="V10" t="inlineStr"/>
+      <c r="W10" t="n">
+        <v>-256.8290392545429</v>
+      </c>
+      <c r="X10" t="n">
+        <v>-167.7548004341224</v>
+      </c>
+      <c r="Y10" t="n">
+        <v>306.761843248315</v>
+      </c>
+      <c r="Z10" t="n">
+        <v>-194.2102282909209</v>
+      </c>
+      <c r="AA10" t="n">
+        <v>-156.8099907686192</v>
+      </c>
+      <c r="AB10" t="n">
+        <v>249.6136734589394</v>
+      </c>
+      <c r="AC10" t="n">
+        <v>92.1884208810102</v>
+      </c>
+      <c r="AD10" t="n">
+        <v>28.1971264084378</v>
+      </c>
+      <c r="AE10" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>